<commit_message>
feat(docs): added pdf docs for technical and user guide
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/4PROJ - User Stories.xlsx
+++ b/docs/fonctionnalites/4PROJ - User Stories.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="203">
   <si>
     <t>Epic ID</t>
   </si>
@@ -177,87 +177,87 @@
     <t xml:space="preserve">Connexion OAuth2 (interfacage) </t>
   </si>
   <si>
+    <t>US-04</t>
+  </si>
+  <si>
+    <t>Gestion JWT &amp; sessions</t>
+  </si>
+  <si>
+    <t>US-05</t>
+  </si>
+  <si>
+    <t>Hachage et vérification des mots de passe</t>
+  </si>
+  <si>
+    <t>US-06</t>
+  </si>
+  <si>
+    <t>Déconnexion utilisateur</t>
+  </si>
+  <si>
+    <t>US-07</t>
+  </si>
+  <si>
+    <t>Connexion via OAuth2 (GitHub, Microsoft, Google)</t>
+  </si>
+  <si>
+    <t>US-08</t>
+  </si>
+  <si>
+    <t>Création automatique d’un compte local après OAuth</t>
+  </si>
+  <si>
+    <t>US-09</t>
+  </si>
+  <si>
+    <t>Modification profil utilisateur</t>
+  </si>
+  <si>
+    <t>Should</t>
+  </si>
+  <si>
+    <t>US-10</t>
+  </si>
+  <si>
+    <t>Changement de mot de passe(NonOAuth2)</t>
+  </si>
+  <si>
+    <t>US-11</t>
+  </si>
+  <si>
+    <t>Client Web connecté API</t>
+  </si>
+  <si>
+    <t>US-12</t>
+  </si>
+  <si>
+    <t>Sécurisation des routes API par authentification</t>
+  </si>
+  <si>
+    <t>À vérifier sur toutes les routes à la fin avec la documentation à faire</t>
+  </si>
+  <si>
+    <t>US-13</t>
+  </si>
+  <si>
+    <t>Gestion des droits d’accès par ressource</t>
+  </si>
+  <si>
+    <t>US-14</t>
+  </si>
+  <si>
+    <t>Protection contre accès non autorisés</t>
+  </si>
+  <si>
+    <t>US-15</t>
+  </si>
+  <si>
+    <t>Gestion centralisée des erreurs API</t>
+  </si>
+  <si>
     <t>NOK</t>
   </si>
   <si>
-    <t>US-04</t>
-  </si>
-  <si>
-    <t>Gestion JWT &amp; sessions</t>
-  </si>
-  <si>
-    <t>US-05</t>
-  </si>
-  <si>
-    <t>Hachage et vérification des mots de passe</t>
-  </si>
-  <si>
-    <t>US-06</t>
-  </si>
-  <si>
-    <t>Déconnexion utilisateur</t>
-  </si>
-  <si>
-    <t>US-07</t>
-  </si>
-  <si>
-    <t>Connexion via OAuth2 (GitHub, Microsoft, Google)</t>
-  </si>
-  <si>
-    <t>US-08</t>
-  </si>
-  <si>
-    <t>Création automatique d’un compte local après OAuth</t>
-  </si>
-  <si>
-    <t>US-09</t>
-  </si>
-  <si>
-    <t>Modification profil utilisateur</t>
-  </si>
-  <si>
-    <t>Should</t>
-  </si>
-  <si>
-    <t>US-10</t>
-  </si>
-  <si>
-    <t>Changement de mot de passe(NonOAuth2)</t>
-  </si>
-  <si>
-    <t>US-11</t>
-  </si>
-  <si>
-    <t>Client Web connecté API</t>
-  </si>
-  <si>
-    <t>US-12</t>
-  </si>
-  <si>
-    <t>Sécurisation des routes API par authentification</t>
-  </si>
-  <si>
-    <t>À vérifier sur toutes les routes à la fin avec la documentation à faire</t>
-  </si>
-  <si>
-    <t>US-13</t>
-  </si>
-  <si>
-    <t>Gestion des droits d’accès par ressource</t>
-  </si>
-  <si>
-    <t>US-14</t>
-  </si>
-  <si>
-    <t>Protection contre accès non autorisés</t>
-  </si>
-  <si>
-    <t>US-15</t>
-  </si>
-  <si>
-    <t>Gestion centralisée des erreurs API</t>
-  </si>
-  <si>
     <t>US-16</t>
   </si>
   <si>
@@ -268,9 +268,6 @@
   </si>
   <si>
     <t>Mise en place du serveur applicatif</t>
-  </si>
-  <si>
-    <t>À faire ave cOVH</t>
   </si>
   <si>
     <t>US-18</t>
@@ -644,10 +641,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="29">
     <font>
@@ -725,24 +722,23 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
@@ -773,31 +769,40 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFA7D00"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -823,6 +828,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
@@ -830,32 +843,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF9C0006"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -888,7 +885,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -900,19 +933,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -924,49 +975,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -978,55 +987,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1044,6 +1005,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1056,7 +1047,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1068,7 +1065,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1330,6 +1327,30 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
@@ -1339,11 +1360,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1363,32 +1390,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1404,25 +1410,16 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
+      <left style="thin">
         <color rgb="FF3F3F3F"/>
       </left>
-      <right style="double">
+      <right style="thin">
         <color rgb="FF3F3F3F"/>
       </right>
-      <top style="double">
+      <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
+      <bottom style="thin">
         <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
@@ -1430,142 +1427,142 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="23" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2639,7 +2636,7 @@
         <v>47</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G4" s="32" t="s">
         <v>48</v>
@@ -2648,10 +2645,10 @@
     </row>
     <row r="5" customHeight="1" spans="1:8">
       <c r="A5" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>54</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>55</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>3</v>
@@ -2672,10 +2669,10 @@
     </row>
     <row r="6" customHeight="1" spans="1:8">
       <c r="A6" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>56</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>57</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>3</v>
@@ -2696,10 +2693,10 @@
     </row>
     <row r="7" customHeight="1" spans="1:8">
       <c r="A7" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>58</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>59</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>3</v>
@@ -2720,10 +2717,10 @@
     </row>
     <row r="8" customHeight="1" spans="1:8">
       <c r="A8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="16" t="s">
         <v>60</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>61</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>3</v>
@@ -2744,10 +2741,10 @@
     </row>
     <row r="9" customHeight="1" spans="1:8">
       <c r="A9" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="16" t="s">
         <v>62</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>63</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>3</v>
@@ -2768,16 +2765,16 @@
     </row>
     <row r="10" customHeight="1" spans="1:8">
       <c r="A10" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>64</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>65</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E10" s="45" t="s">
         <v>47</v>
@@ -2792,10 +2789,10 @@
     </row>
     <row r="11" customHeight="1" spans="1:8">
       <c r="A11" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="23" t="s">
         <v>67</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>68</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>21</v>
@@ -2816,10 +2813,10 @@
     </row>
     <row r="12" customHeight="1" spans="1:8">
       <c r="A12" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>69</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>70</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>24</v>
@@ -2840,10 +2837,10 @@
     </row>
     <row r="13" customHeight="1" spans="1:8">
       <c r="A13" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="27" t="s">
         <v>71</v>
-      </c>
-      <c r="B13" s="27" t="s">
-        <v>72</v>
       </c>
       <c r="C13" s="27" t="s">
         <v>27</v>
@@ -2861,15 +2858,15 @@
         <v>48</v>
       </c>
       <c r="H13" s="50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="1:8">
       <c r="A14" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="30" t="s">
         <v>74</v>
-      </c>
-      <c r="B14" s="30" t="s">
-        <v>75</v>
       </c>
       <c r="C14" s="30" t="s">
         <v>27</v>
@@ -2890,10 +2887,10 @@
     </row>
     <row r="15" customHeight="1" spans="1:8">
       <c r="A15" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="32" t="s">
         <v>76</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>77</v>
       </c>
       <c r="C15" s="32" t="s">
         <v>27</v>
@@ -2911,30 +2908,30 @@
         <v>48</v>
       </c>
       <c r="H15" s="44" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="1:8">
       <c r="A16" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="30" t="s">
         <v>78</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>79</v>
       </c>
       <c r="C16" s="30" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E16" s="49" t="s">
         <v>47</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="G16" s="32" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="H16" s="43"/>
     </row>
@@ -2979,21 +2976,19 @@
         <v>47</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="G18" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="H18" s="44" t="s">
-        <v>84</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="H18" s="44"/>
     </row>
     <row r="19" customHeight="1" spans="1:8">
       <c r="A19" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="30" t="s">
         <v>85</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>86</v>
       </c>
       <c r="C19" s="30" t="s">
         <v>30</v>
@@ -3014,10 +3009,10 @@
     </row>
     <row r="20" customHeight="1" spans="1:8">
       <c r="A20" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="32" t="s">
         <v>87</v>
-      </c>
-      <c r="B20" s="32" t="s">
-        <v>88</v>
       </c>
       <c r="C20" s="32" t="s">
         <v>30</v>
@@ -3035,15 +3030,15 @@
         <v>48</v>
       </c>
       <c r="H20" s="44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:8">
       <c r="A21" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="35" t="s">
         <v>90</v>
-      </c>
-      <c r="B21" s="35" t="s">
-        <v>91</v>
       </c>
       <c r="C21" s="35" t="s">
         <v>30</v>
@@ -3064,10 +3059,10 @@
     </row>
     <row r="22" customHeight="1" spans="1:8">
       <c r="A22" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="B22" s="27" t="s">
         <v>92</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>93</v>
       </c>
       <c r="C22" s="27" t="s">
         <v>33</v>
@@ -3079,21 +3074,21 @@
         <v>47</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G22" s="32" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="H22" s="50" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" customHeight="1" spans="1:8">
       <c r="A23" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="30" t="s">
         <v>95</v>
-      </c>
-      <c r="B23" s="30" t="s">
-        <v>96</v>
       </c>
       <c r="C23" s="30" t="s">
         <v>33</v>
@@ -3105,21 +3100,21 @@
         <v>47</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G23" s="32" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="H23" s="50" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="1:8">
       <c r="A24" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="23" t="s">
         <v>97</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>98</v>
       </c>
       <c r="C24" s="23" t="s">
         <v>33</v>
@@ -3140,106 +3135,106 @@
     </row>
     <row r="25" customHeight="1" spans="1:8">
       <c r="A25" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>99</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>100</v>
       </c>
       <c r="C25" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D25" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="E25" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="E25" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="F25" s="16" t="s">
-        <v>102</v>
-      </c>
       <c r="G25" s="32" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="H25" s="46"/>
     </row>
     <row r="26" customHeight="1" spans="1:8">
       <c r="A26" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B26" s="30" t="s">
         <v>103</v>
-      </c>
-      <c r="B26" s="30" t="s">
-        <v>104</v>
       </c>
       <c r="C26" s="30" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E26" s="42" t="s">
         <v>47</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="G26" s="32" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="H26" s="43"/>
     </row>
     <row r="27" customHeight="1" spans="1:8">
       <c r="A27" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="B27" s="32" t="s">
         <v>105</v>
-      </c>
-      <c r="B27" s="32" t="s">
-        <v>106</v>
       </c>
       <c r="C27" s="32" t="s">
         <v>9</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E27" s="52" t="s">
         <v>47</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="G27" s="32" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="H27" s="44"/>
     </row>
     <row r="28" customHeight="1" spans="1:8">
       <c r="A28" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="B28" s="30" t="s">
         <v>107</v>
-      </c>
-      <c r="B28" s="30" t="s">
-        <v>108</v>
       </c>
       <c r="C28" s="30" t="s">
         <v>9</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E28" s="42" t="s">
         <v>47</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="G28" s="32" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="H28" s="43"/>
     </row>
     <row r="29" ht="73" customHeight="1" spans="1:8">
       <c r="A29" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>109</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>110</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>6</v>
@@ -3257,15 +3252,15 @@
         <v>48</v>
       </c>
       <c r="H29" s="53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:8">
       <c r="A30" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>112</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>113</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>6</v>
@@ -3283,15 +3278,15 @@
         <v>48</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="1:7">
       <c r="A31" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="12" t="s">
         <v>115</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>116</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>15</v>
@@ -3311,10 +3306,10 @@
     </row>
     <row r="32" customHeight="1" spans="1:7">
       <c r="A32" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="12" t="s">
         <v>117</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>118</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>6</v>
@@ -3334,10 +3329,10 @@
     </row>
     <row r="33" customHeight="1" spans="1:7">
       <c r="A33" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>119</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>120</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>15</v>
@@ -3357,16 +3352,16 @@
     </row>
     <row r="34" customHeight="1" spans="1:8">
       <c r="A34" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="B34" s="12" t="s">
         <v>121</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>122</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E34" s="52" t="s">
         <v>47</v>
@@ -3378,15 +3373,15 @@
         <v>48</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" customHeight="1" spans="1:7">
       <c r="A35" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>124</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>125</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>6</v>
@@ -3406,10 +3401,10 @@
     </row>
     <row r="36" customHeight="1" spans="1:7">
       <c r="A36" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="B36" s="12" t="s">
         <v>126</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>127</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>6</v>
@@ -3429,10 +3424,10 @@
     </row>
     <row r="37" customHeight="1" spans="1:7">
       <c r="A37" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>128</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>129</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>6</v>
@@ -3452,10 +3447,10 @@
     </row>
     <row r="38" customHeight="1" spans="1:8">
       <c r="A38" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="12" t="s">
         <v>130</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>131</v>
       </c>
       <c r="C38" s="12" t="s">
         <v>6</v>
@@ -3473,15 +3468,15 @@
         <v>48</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" customHeight="1" spans="1:8">
       <c r="A39" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="B39" s="12" t="s">
         <v>132</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>133</v>
       </c>
       <c r="C39" s="12" t="s">
         <v>6</v>
@@ -3499,15 +3494,15 @@
         <v>48</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="40" customHeight="1" spans="1:7">
       <c r="A40" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="B40" s="12" t="s">
         <v>135</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>136</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>6</v>
@@ -3527,16 +3522,16 @@
     </row>
     <row r="41" customHeight="1" spans="1:7">
       <c r="A41" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B41" s="12" t="s">
         <v>137</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>138</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>6</v>
       </c>
       <c r="D41" s="39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E41" s="52" t="s">
         <v>47</v>
@@ -3550,10 +3545,10 @@
     </row>
     <row r="42" customHeight="1" spans="1:7">
       <c r="A42" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="B42" s="12" t="s">
         <v>139</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>140</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>9</v>
@@ -3573,16 +3568,16 @@
     </row>
     <row r="43" customHeight="1" spans="1:8">
       <c r="A43" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>141</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>142</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>9</v>
       </c>
       <c r="D43" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E43" s="52" t="s">
         <v>47</v>
@@ -3594,15 +3589,15 @@
         <v>48</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="44" customHeight="1" spans="1:7">
       <c r="A44" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="B44" s="12" t="s">
         <v>144</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>145</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>9</v>
@@ -3622,10 +3617,10 @@
     </row>
     <row r="45" customHeight="1" spans="1:7">
       <c r="A45" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B45" s="12" t="s">
         <v>146</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>147</v>
       </c>
       <c r="C45" s="12" t="s">
         <v>9</v>
@@ -3645,10 +3640,10 @@
     </row>
     <row r="46" customHeight="1" spans="1:8">
       <c r="A46" s="31" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46" s="12" t="s">
         <v>148</v>
-      </c>
-      <c r="B46" s="12" t="s">
-        <v>149</v>
       </c>
       <c r="C46" s="12" t="s">
         <v>9</v>
@@ -3666,15 +3661,15 @@
         <v>48</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="1:7">
       <c r="A47" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B47" s="12" t="s">
         <v>151</v>
-      </c>
-      <c r="B47" s="12" t="s">
-        <v>152</v>
       </c>
       <c r="C47" s="12" t="s">
         <v>9</v>
@@ -3694,10 +3689,10 @@
     </row>
     <row r="48" customHeight="1" spans="1:8">
       <c r="A48" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="B48" s="12" t="s">
         <v>153</v>
-      </c>
-      <c r="B48" s="12" t="s">
-        <v>154</v>
       </c>
       <c r="C48" s="12" t="s">
         <v>9</v>
@@ -3712,18 +3707,18 @@
         <v>48</v>
       </c>
       <c r="G48" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="H48" s="12" t="s">
         <v>155</v>
-      </c>
-      <c r="H48" s="12" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="49" customHeight="1" spans="1:7">
       <c r="A49" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B49" s="12" t="s">
         <v>157</v>
-      </c>
-      <c r="B49" s="12" t="s">
-        <v>158</v>
       </c>
       <c r="C49" s="12" t="s">
         <v>12</v>
@@ -3738,15 +3733,15 @@
         <v>48</v>
       </c>
       <c r="G49" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="50" ht="85" customHeight="1" spans="1:8">
       <c r="A50" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="B50" s="12" t="s">
         <v>159</v>
-      </c>
-      <c r="B50" s="12" t="s">
-        <v>160</v>
       </c>
       <c r="C50" s="12" t="s">
         <v>12</v>
@@ -3764,21 +3759,21 @@
         <v>48</v>
       </c>
       <c r="H50" s="53" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" customHeight="1" spans="1:7">
       <c r="A51" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B51" s="12" t="s">
         <v>162</v>
-      </c>
-      <c r="B51" s="12" t="s">
-        <v>163</v>
       </c>
       <c r="C51" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D51" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E51" s="52" t="s">
         <v>47</v>
@@ -3792,16 +3787,16 @@
     </row>
     <row r="52" customHeight="1" spans="1:7">
       <c r="A52" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="B52" s="12" t="s">
         <v>164</v>
-      </c>
-      <c r="B52" s="12" t="s">
-        <v>165</v>
       </c>
       <c r="C52" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D52" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E52" s="52" t="s">
         <v>47</v>
@@ -3815,10 +3810,10 @@
     </row>
     <row r="53" customHeight="1" spans="1:7">
       <c r="A53" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="B53" s="12" t="s">
         <v>166</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>167</v>
       </c>
       <c r="C53" s="12" t="s">
         <v>18</v>
@@ -3838,10 +3833,10 @@
     </row>
     <row r="54" customHeight="1" spans="1:7">
       <c r="A54" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B54" s="12" t="s">
         <v>168</v>
-      </c>
-      <c r="B54" s="12" t="s">
-        <v>169</v>
       </c>
       <c r="C54" s="12" t="s">
         <v>18</v>
@@ -3861,10 +3856,10 @@
     </row>
     <row r="55" customHeight="1" spans="1:7">
       <c r="A55" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="B55" s="12" t="s">
         <v>170</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>171</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>18</v>
@@ -3884,10 +3879,10 @@
     </row>
     <row r="56" customHeight="1" spans="1:7">
       <c r="A56" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="B56" s="12" t="s">
         <v>172</v>
-      </c>
-      <c r="B56" s="12" t="s">
-        <v>173</v>
       </c>
       <c r="C56" s="12" t="s">
         <v>18</v>
@@ -3907,10 +3902,10 @@
     </row>
     <row r="57" customHeight="1" spans="1:7">
       <c r="A57" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B57" s="12" t="s">
         <v>174</v>
-      </c>
-      <c r="B57" s="12" t="s">
-        <v>175</v>
       </c>
       <c r="C57" s="12" t="s">
         <v>6</v>
@@ -3930,10 +3925,10 @@
     </row>
     <row r="58" customHeight="1" spans="1:7">
       <c r="A58" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B58" s="12" t="s">
         <v>176</v>
-      </c>
-      <c r="B58" s="12" t="s">
-        <v>177</v>
       </c>
       <c r="C58" s="12" t="s">
         <v>6</v>
@@ -3953,10 +3948,10 @@
     </row>
     <row r="59" customHeight="1" spans="1:8">
       <c r="A59" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="B59" s="12" t="s">
         <v>178</v>
-      </c>
-      <c r="B59" s="12" t="s">
-        <v>179</v>
       </c>
       <c r="C59" s="40" t="s">
         <v>24</v>
@@ -3968,21 +3963,21 @@
         <v>47</v>
       </c>
       <c r="F59" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G59" s="12" t="s">
         <v>48</v>
       </c>
       <c r="H59" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="60" customHeight="1" spans="1:8">
       <c r="A60" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="B60" s="12" t="s">
         <v>181</v>
-      </c>
-      <c r="B60" s="12" t="s">
-        <v>182</v>
       </c>
       <c r="C60" s="40" t="s">
         <v>24</v>
@@ -3994,21 +3989,21 @@
         <v>47</v>
       </c>
       <c r="F60" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G60" s="12" t="s">
         <v>48</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" customHeight="1" spans="1:7">
       <c r="A61" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B61" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="B61" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="C61" s="40" t="s">
         <v>24</v>
@@ -4020,7 +4015,7 @@
         <v>47</v>
       </c>
       <c r="F61" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G61" s="12" t="s">
         <v>48</v>
@@ -4028,10 +4023,10 @@
     </row>
     <row r="62" customHeight="1" spans="1:7">
       <c r="A62" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="B62" s="12" t="s">
         <v>186</v>
-      </c>
-      <c r="B62" s="12" t="s">
-        <v>187</v>
       </c>
       <c r="C62" s="40" t="s">
         <v>9</v>
@@ -4051,10 +4046,10 @@
     </row>
     <row r="63" customHeight="1" spans="1:7">
       <c r="A63" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B63" s="12" t="s">
         <v>188</v>
-      </c>
-      <c r="B63" s="12" t="s">
-        <v>189</v>
       </c>
       <c r="C63" s="40" t="s">
         <v>9</v>
@@ -4066,7 +4061,7 @@
         <v>47</v>
       </c>
       <c r="F63" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G63" s="12" t="s">
         <v>48</v>
@@ -4074,10 +4069,10 @@
     </row>
     <row r="64" customHeight="1" spans="1:7">
       <c r="A64" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="B64" s="12" t="s">
         <v>190</v>
-      </c>
-      <c r="B64" s="12" t="s">
-        <v>191</v>
       </c>
       <c r="C64" s="40" t="s">
         <v>9</v>
@@ -4097,16 +4092,16 @@
     </row>
     <row r="65" customHeight="1" spans="1:7">
       <c r="A65" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B65" s="12" t="s">
         <v>192</v>
-      </c>
-      <c r="B65" s="12" t="s">
-        <v>193</v>
       </c>
       <c r="C65" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D65" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E65" s="52" t="s">
         <v>47</v>
@@ -5440,17 +5435,17 @@
     <row r="1" ht="50.25" customHeight="1" spans="1:4">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4">
       <c r="A2" s="4"/>
       <c r="B2" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="6" t="s">
@@ -5460,11 +5455,11 @@
     <row r="3" ht="30" customHeight="1" spans="1:4">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4">
@@ -5474,23 +5469,23 @@
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:4">
       <c r="A5" s="4"/>
       <c r="B5" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:4">
       <c r="A6" s="4"/>
       <c r="B6" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="8"/>
@@ -5498,19 +5493,19 @@
     <row r="7" ht="30" customHeight="1" spans="1:4">
       <c r="A7" s="9"/>
       <c r="B7" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="10"/>
     </row>
     <row r="8" spans="2:2">
       <c r="B8" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="2:2">
       <c r="B9" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="2:2">

</xml_diff>